<commit_message>
updated for march 5th
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="551" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE9356E6-A232-44A3-B93C-904FC1C387E1}"/>
+  <xr:revisionPtr revIDLastSave="553" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE6CF80F-296E-4359-BC23-66D167DA63B8}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeGames" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="69">
   <si>
     <t>manler</t>
   </si>
@@ -582,6 +582,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1471,9 +1475,9 @@
         <f>IF(OR(B8 = "UNPLAYED", B8 = "XXX"), B8, -1* B8)</f>
         <v>UNPLAYED</v>
       </c>
-      <c r="I2" s="1" t="str">
+      <c r="I2" s="1">
         <f>IF(OR(B9 = "UNPLAYED", B9 = "XXX"), B9, -1* B9)</f>
-        <v>UNPLAYED</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="str">
         <f>IF(OR(B10 = "UNPLAYED", B10 = "XXX"), B10, -1* B10)</f>
@@ -1502,9 +1506,9 @@
         <f>IF(OR(C5 = "UNPLAYED", C5 = "XXX"), C5, -1* C5)</f>
         <v>UNPLAYED</v>
       </c>
-      <c r="F3" s="1" t="str">
+      <c r="F3" s="1">
         <f>IF(OR(C6 = "UNPLAYED", C6 = "XXX"), C6, -1* C6)</f>
-        <v>UNPLAYED</v>
+        <v>-60</v>
       </c>
       <c r="G3" s="1" t="str">
         <f>IF(OR(C7 = "UNPLAYED", C7 = "XXX"), C7, -1* C7)</f>
@@ -1617,8 +1621,8 @@
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>4</v>
+      <c r="C6" s="3">
+        <v>60</v>
       </c>
       <c r="D6" s="3">
         <v>100</v>
@@ -1731,8 +1735,8 @@
       <c r="A9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>4</v>
+      <c r="B9" s="3">
+        <v>-100</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
update 4th to last session
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="684" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{733BFF86-C76A-4305-ACB2-1FBEC985CAF7}"/>
+  <xr:revisionPtr revIDLastSave="705" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52226454-6F80-44B5-94A8-946EED17CC40}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeGames" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="71">
   <si>
     <t>manler</t>
   </si>
@@ -249,6 +249,12 @@
   </si>
   <si>
     <t>away TRON won by 100</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>-F</t>
   </si>
 </sst>
 </file>
@@ -356,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -379,119 +385,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCD094"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="30">
     <dxf>
       <font>
         <b val="0"/>
@@ -1221,9 +1122,9 @@
         <f>IF(OR(C9 = "UNPLAYED", C9 = "XXX"), C9, IF(C9 = "F", "-F", IF(C9 = "-F", "F", -1*C9)))</f>
         <v>XXX</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="J3" s="4">
         <f>IF(OR(C10 = "UNPLAYED", C10 = "XXX"), C10, IF(C10 = "F", "-F", IF(C10 = "-F", "F", -1*C10)))</f>
-        <v>UNPLAYED</v>
+        <v>-75</v>
       </c>
       <c r="K3" s="4" t="str">
         <f>IF(OR(C11 = "UNPLAYED", C11 = "XXX"), C11, IF(C11 = "F", "-F", IF(C11 = "-F", "F", -1*C11)))</f>
@@ -1481,8 +1382,8 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>4</v>
+      <c r="C10" s="3">
+        <v>75</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>4</v>
@@ -1570,43 +1471,43 @@
       <c r="K13" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B9:B10 O10:Q12 O3:O9 G6:K6 H7:K7 I8:K8 K10 J9:K9 B2:K5">
-    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
+  <conditionalFormatting sqref="B6:D7 F6:H7">
+    <cfRule type="cellIs" dxfId="29" priority="13" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="14" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:D7 B8:H8 F6:H7">
-    <cfRule type="cellIs" dxfId="39" priority="13" operator="equal">
+  <conditionalFormatting sqref="B2:K5 O3:O9 G6:K6 H7:K7 B8:K8 J9:K9 B9:B10 K10 O10:Q12">
+    <cfRule type="cellIs" dxfId="27" priority="7" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="8" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="cellIs" dxfId="37" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="9" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="10" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7">
-    <cfRule type="cellIs" dxfId="35" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="6" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11">
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="4" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1671,7 +1572,7 @@
       </c>
       <c r="D2" s="4" t="str">
         <f>IF(OR(B4 = "UNPLAYED", B4 = "XXX"), B4, IF(B4 = "F", "-F", IF(B4 = "-F", "F", -1*B4)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="E2" s="4">
         <f>IF(OR(B5 = "UNPLAYED", B5 = "XXX"), B5, IF(B5 = "F", "-F", IF(B5 = "-F", "F", -1*B5)))</f>
@@ -1687,7 +1588,7 @@
       </c>
       <c r="H2" s="4" t="str">
         <f>IF(OR(B8 = "UNPLAYED", B8 = "XXX"), B8, IF(B8 = "F", "-F", IF(B8 = "-F", "F", -1*B8)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="I2" s="4">
         <f>IF(OR(B9 = "UNPLAYED", B9 = "XXX"), B9, IF(B9 = "F", "-F", IF(B9 = "-F", "F", -1*B9)))</f>
@@ -1718,7 +1619,7 @@
       </c>
       <c r="E3" s="4" t="str">
         <f>IF(OR(C5 = "UNPLAYED", C5 = "XXX"), C5, IF(C5 = "F", "-F", IF(C5 = "-F", "F", -1*C5)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="F3" s="4">
         <f>IF(OR(C6 = "UNPLAYED", C6 = "XXX"), C6, IF(C6 = "F", "-F", IF(C6 = "-F", "F", -1*C6)))</f>
@@ -1726,7 +1627,7 @@
       </c>
       <c r="G3" s="4" t="str">
         <f>IF(OR(C7 = "UNPLAYED", C7 = "XXX"), C7, IF(C7 = "F", "-F", IF(C7 = "-F", "F", -1*C7)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="H3" s="4" t="str">
         <f>IF(OR(C8 = "UNPLAYED", C8 = "XXX"), C8, IF(C8 = "F", "-F", IF(C8 = "-F", "F", -1*C8)))</f>
@@ -1736,21 +1637,21 @@
         <f>IF(OR(C9 = "UNPLAYED", C9 = "XXX"), C9, IF(C9 = "F", "-F", IF(C9 = "-F", "F", -1*C9)))</f>
         <v>XXX</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="J3" s="4">
         <f>IF(OR(C10 = "UNPLAYED", C10 = "XXX"), C10, IF(C10 = "F", "-F", IF(C10 = "-F", "F", -1*C10)))</f>
-        <v>UNPLAYED</v>
+        <v>-45</v>
       </c>
       <c r="K3" s="4" t="str">
         <f>IF(OR(C11 = "UNPLAYED", C11 = "XXX"), C11, IF(C11 = "F", "-F", IF(C11 = "-F", "F", -1*C11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>4</v>
+      <c r="B4" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -1780,7 +1681,7 @@
       </c>
       <c r="J4" s="4" t="str">
         <f>IF(OR(D10 = "UNPLAYED", D10 = "XXX"), D10, IF(D10 = "F", "-F", IF(D10 = "-F", "F", -1*D10)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="K4" s="4" t="str">
         <f>IF(OR(D11 = "UNPLAYED", D11 = "XXX"), D11, IF(D11 = "F", "-F", IF(D11 = "-F", "F", -1*D11)))</f>
@@ -1794,8 +1695,8 @@
       <c r="B5" s="3">
         <v>-100</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>4</v>
+      <c r="C5" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>4</v>
@@ -1817,7 +1718,7 @@
       </c>
       <c r="I5" s="4" t="str">
         <f>IF(OR(E9 = "UNPLAYED", E9 = "XXX"), E9, IF(E9 = "F", "-F", IF(E9 = "-F", "F", -1*E9)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="J5" s="4" t="str">
         <f>IF(OR(E10 = "UNPLAYED", E10 = "XXX"), E10, IF(E10 = "F", "-F", IF(E10 = "-F", "F", -1*E10)))</f>
@@ -1855,9 +1756,9 @@
         <f>IF(OR(F8 = "UNPLAYED", F8 = "XXX"), F8, IF(F8 = "F", "-F", IF(F8 = "-F", "F", -1*F8)))</f>
         <v>UNPLAYED</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="4">
         <f>IF(OR(F9 = "UNPLAYED", F9 = "XXX"), F9, IF(F9 = "F", "-F", IF(F9 = "-F", "F", -1*F9)))</f>
-        <v>UNPLAYED</v>
+        <v>-70</v>
       </c>
       <c r="J6" s="4">
         <f>IF(OR(F10 = "UNPLAYED", F10 = "XXX"), F10, IF(F10 = "F", "-F", IF(F10 = "-F", "F", -1*F10)))</f>
@@ -1865,7 +1766,7 @@
       </c>
       <c r="K6" s="4" t="str">
         <f>IF(OR(F11 = "UNPLAYED", F11 = "XXX"), F11, IF(F11 = "F", "-F", IF(F11 = "-F", "F", -1*F11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="25.5" x14ac:dyDescent="0.55000000000000004">
@@ -1875,8 +1776,8 @@
       <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>4</v>
+      <c r="C7" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>4</v>
@@ -1911,8 +1812,8 @@
       <c r="A8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>4</v>
+      <c r="B8" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>3</v>
@@ -1938,7 +1839,7 @@
       </c>
       <c r="J8" s="4" t="str">
         <f>IF(OR(H10 = "UNPLAYED", H10 = "XXX"), H10, IF(H10 = "F", "-F", IF(H10 = "-F", "F", -1*H10)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="K8" s="4" t="str">
         <f>IF(OR(H11 = "UNPLAYED", H11 = "XXX"), H11, IF(H11 = "F", "-F", IF(H11 = "-F", "F", -1*H11)))</f>
@@ -1959,10 +1860,10 @@
         <v>4</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
+      </c>
+      <c r="F9" s="3">
+        <v>70</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>3</v>
@@ -1973,9 +1874,9 @@
       <c r="I9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J9" s="4" t="str">
+      <c r="J9" s="4">
         <f>IF(OR(I10 = "UNPLAYED", I10 = "XXX"), I10, IF(I10 = "F", "-F", IF(I10 = "-F", "F", -1*I10)))</f>
-        <v>UNPLAYED</v>
+        <v>-100</v>
       </c>
       <c r="K9" s="4">
         <f>IF(OR(I11 = "UNPLAYED", I11 = "XXX"), I11, IF(I11 = "F", "-F", IF(I11 = "-F", "F", -1*I11)))</f>
@@ -1990,11 +1891,11 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>4</v>
+      <c r="C10" s="3">
+        <v>45</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>3</v>
@@ -2006,10 +1907,10 @@
         <v>4</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
+      </c>
+      <c r="I10" s="3">
+        <v>100</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>3</v>
@@ -2027,8 +1928,8 @@
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>4</v>
+      <c r="C11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>3</v>
@@ -2036,8 +1937,8 @@
       <c r="E11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>4</v>
+      <c r="F11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>3</v>
@@ -2083,70 +1984,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="cellIs" dxfId="31" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="23" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="24" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:E5 B6:D7 F7:G7 B8:H8 B2 B3:C3 B4:D4 F6">
-    <cfRule type="cellIs" dxfId="29" priority="33" operator="equal">
+  <conditionalFormatting sqref="B6:D7">
+    <cfRule type="cellIs" dxfId="17" priority="33" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="34" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="cellIs" dxfId="27" priority="29" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="30" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
-    <cfRule type="cellIs" dxfId="25" priority="25" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="26" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11">
-    <cfRule type="cellIs" dxfId="23" priority="27" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="28" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:K2">
-    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:K3">
-    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E4:K4">
-    <cfRule type="cellIs" dxfId="17" priority="17" operator="equal">
-      <formula>"UNPLAYED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="18" operator="equal">
-      <formula>"XXX"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F5:K5">
+  <conditionalFormatting sqref="B2:K5">
     <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
@@ -2154,23 +2007,23 @@
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G6:K6">
-    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+  <conditionalFormatting sqref="B8:K8">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G6:H6">
-    <cfRule type="cellIs" dxfId="11" priority="13" operator="equal">
+  <conditionalFormatting sqref="C9">
+    <cfRule type="cellIs" dxfId="11" priority="29" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="30" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:K7">
+  <conditionalFormatting sqref="E7:K7">
     <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
@@ -2178,19 +2031,19 @@
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7">
-    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
+  <conditionalFormatting sqref="F6:K6">
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I8:K8">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+  <conditionalFormatting sqref="G11">
+    <cfRule type="cellIs" dxfId="5" priority="27" operator="equal">
       <formula>"UNPLAYED"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="28" operator="equal">
       <formula>"XXX"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
updated for most recent march madness
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="717" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E67BB088-1743-42F9-A9B4-40297A48C787}"/>
+  <xr:revisionPtr revIDLastSave="737" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD69A10F-27A1-4214-A3EF-AAA670CC34DE}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
@@ -19,7 +19,8 @@
     <sheet name="TeamInfo" sheetId="3" r:id="rId4"/>
     <sheet name="AwayGamesBig" sheetId="6" r:id="rId5"/>
     <sheet name="notes" sheetId="5" r:id="rId6"/>
-    <sheet name="GameCalculator" sheetId="4" r:id="rId7"/>
+    <sheet name="spring tourney" sheetId="8" r:id="rId7"/>
+    <sheet name="GameCalculator" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="77">
   <si>
     <t>manler</t>
   </si>
@@ -255,6 +256,24 @@
   </si>
   <si>
     <t>-F</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>Na'ama</t>
+  </si>
+  <si>
+    <t>Team name</t>
+  </si>
+  <si>
+    <t>player</t>
+  </si>
+  <si>
+    <t>Nick</t>
+  </si>
+  <si>
+    <t>The Sweatshop</t>
   </si>
 </sst>
 </file>
@@ -1102,9 +1121,9 @@
         <f>IF(OR(C4 = "UNPLAYED", C4 = "XXX"), C4, IF(C4 = "F", "-F", IF(C4 = "-F", "F", -1*C4)))</f>
         <v>60</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="4">
         <f>IF(OR(C5 = "UNPLAYED", C5 = "XXX"), C5, IF(C5 = "F", "-F", IF(C5 = "-F", "F", -1*C5)))</f>
-        <v>F</v>
+        <v>100</v>
       </c>
       <c r="F3" s="4">
         <f>IF(OR(C6 = "UNPLAYED", C6 = "XXX"), C6, IF(C6 = "F", "-F", IF(C6 = "-F", "F", -1*C6)))</f>
@@ -1182,8 +1201,8 @@
       <c r="B5" s="3">
         <v>-95</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>70</v>
+      <c r="C5" s="14">
+        <v>-100</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>4</v>
@@ -3305,6 +3324,59 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCB3BC70-835A-40D4-BE4F-1F491AA8373B}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="9.734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2">
+        <f>COUNTA(A2:A22) + 0.5 * COUNTA(G2:G22)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E89C9DF-CBF0-44E0-B9C4-2CFC23F872E2}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>

<commit_message>
updated the jpFlicks scores
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="737" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD69A10F-27A1-4214-A3EF-AAA670CC34DE}"/>
+  <xr:revisionPtr revIDLastSave="745" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5AD9538-1F51-4AED-9B18-8E36F814BEB6}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="K3" s="4" t="str">
         <f>IF(OR(C11 = "UNPLAYED", C11 = "XXX"), C11, IF(C11 = "F", "-F", IF(C11 = "-F", "F", -1*C11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="O3" s="4"/>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="E4" s="4" t="str">
         <f>IF(OR(D5 = "UNPLAYED", D5 = "XXX"), D5, IF(D5 = "F", "-F", IF(D5 = "-F", "F", -1*D5)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="F4" s="4">
         <f>IF(OR(D6 = "UNPLAYED", D6 = "XXX"), D6, IF(D6 = "F", "-F", IF(D6 = "-F", "F", -1*D6)))</f>
@@ -1205,7 +1205,7 @@
         <v>-100</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>3</v>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="G5" s="4" t="str">
         <f>IF(OR(E7 = "UNPLAYED", E7 = "XXX"), E7, IF(E7 = "F", "-F", IF(E7 = "-F", "F", -1*E7)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="H5" s="4">
         <f>IF(OR(E8 = "UNPLAYED", E8 = "XXX"), E8, IF(E8 = "F", "-F", IF(E8 = "-F", "F", -1*E8)))</f>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="K5" s="4" t="str">
         <f>IF(OR(E11 = "UNPLAYED", E11 = "XXX"), E11, IF(E11 = "F", "-F", IF(E11 = "-F", "F", -1*E11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="O5" s="4"/>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="K6" s="4" t="str">
         <f>IF(OR(F11 = "UNPLAYED", F11 = "XXX"), F11, IF(F11 = "F", "-F", IF(F11 = "-F", "F", -1*F11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="O6" s="4"/>
     </row>
@@ -1290,8 +1290,8 @@
       <c r="D7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>4</v>
+      <c r="E7" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="F7" s="3">
         <v>40</v>
@@ -1440,17 +1440,17 @@
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>4</v>
+      <c r="C11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>4</v>
+      <c r="E11" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>3</v>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="K2" s="4" t="str">
         <f>IF(OR(B11 = "UNPLAYED", B11 = "XXX"), B11, IF(B11 = "F", "-F", IF(B11 = "-F", "F", -1*B11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="H5" s="4" t="str">
         <f>IF(OR(E8 = "UNPLAYED", E8 = "XXX"), E8, IF(E8 = "F", "-F", IF(E8 = "-F", "F", -1*E8)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="I5" s="4" t="str">
         <f>IF(OR(E9 = "UNPLAYED", E9 = "XXX"), E9, IF(E9 = "F", "-F", IF(E9 = "-F", "F", -1*E9)))</f>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="K5" s="4" t="str">
         <f>IF(OR(E11 = "UNPLAYED", E11 = "XXX"), E11, IF(E11 = "F", "-F", IF(E11 = "-F", "F", -1*E11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
@@ -1840,8 +1840,8 @@
       <c r="D8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>4</v>
+      <c r="E8" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>70</v>
@@ -1944,8 +1944,8 @@
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>4</v>
+      <c r="B11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>70</v>
@@ -1953,8 +1953,8 @@
       <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>4</v>
+      <c r="E11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>70</v>

</xml_diff>

<commit_message>
updated for newest tournament
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="745" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5AD9538-1F51-4AED-9B18-8E36F814BEB6}"/>
+  <xr:revisionPtr revIDLastSave="1075" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EE9663C-5C1F-485F-A47E-524B0EA66088}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="6" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeGames" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="130">
   <si>
     <t>manler</t>
   </si>
@@ -273,7 +273,166 @@
     <t>Nick</t>
   </si>
   <si>
-    <t>The Sweatshop</t>
+    <t>Pill Dickle</t>
+  </si>
+  <si>
+    <t>Nawty</t>
+  </si>
+  <si>
+    <t>Ellie</t>
+  </si>
+  <si>
+    <t>jared</t>
+  </si>
+  <si>
+    <t>likely</t>
+  </si>
+  <si>
+    <t>out</t>
+  </si>
+  <si>
+    <t>katelyn</t>
+  </si>
+  <si>
+    <t>kato</t>
+  </si>
+  <si>
+    <t>Tyler</t>
+  </si>
+  <si>
+    <t>Josh</t>
+  </si>
+  <si>
+    <t>will</t>
+  </si>
+  <si>
+    <t>Lisa</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>XX</t>
+  </si>
+  <si>
+    <t>format</t>
+  </si>
+  <si>
+    <t>rr</t>
+  </si>
+  <si>
+    <t>table</t>
+  </si>
+  <si>
+    <t>rr games</t>
+  </si>
+  <si>
+    <t>table games</t>
+  </si>
+  <si>
+    <t>bracket size</t>
+  </si>
+  <si>
+    <t>total games</t>
+  </si>
+  <si>
+    <t>time per game</t>
+  </si>
+  <si>
+    <t>total time</t>
+  </si>
+  <si>
+    <t>Elyse</t>
+  </si>
+  <si>
+    <t>Anand</t>
+  </si>
+  <si>
+    <t>dbl bracket</t>
+  </si>
+  <si>
+    <t>Anand roomate</t>
+  </si>
+  <si>
+    <t>accelerated rules:</t>
+  </si>
+  <si>
+    <t>each player will only have 4 discs instead of 6</t>
+  </si>
+  <si>
+    <t>shot %</t>
+  </si>
+  <si>
+    <t>accelerated</t>
+  </si>
+  <si>
+    <t>kendall</t>
+  </si>
+  <si>
+    <t>clare</t>
+  </si>
+  <si>
+    <t>accell play in</t>
+  </si>
+  <si>
+    <t>time constraint</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Dina</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>dbl bracket games</t>
+  </si>
+  <si>
+    <t>first to winning by 75 or 4 rounds with minimum of 2 rounds. Goal is for games to last 15 minutes</t>
+  </si>
+  <si>
+    <t>moll ball</t>
+  </si>
+  <si>
+    <t>Shake Shack</t>
+  </si>
+  <si>
+    <t>The Sun also Rises</t>
+  </si>
+  <si>
+    <t>Jenny</t>
+  </si>
+  <si>
+    <t>Upekha</t>
+  </si>
+  <si>
+    <t>Abhishek</t>
+  </si>
+  <si>
+    <t>Frolicc</t>
+  </si>
+  <si>
+    <t>Annie</t>
+  </si>
+  <si>
+    <t>Edger Team</t>
+  </si>
+  <si>
+    <t>Jayhawks</t>
+  </si>
+  <si>
+    <t>This Old Store</t>
+  </si>
+  <si>
+    <t>XXXX</t>
+  </si>
+  <si>
+    <t>Milk and Honey</t>
   </si>
 </sst>
 </file>
@@ -381,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -407,6 +566,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3325,13 +3486,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCB3BC70-835A-40D4-BE4F-1F491AA8373B}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:W22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="9.734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.05078125" customWidth="1"/>
+    <col min="14" max="14" width="10.7890625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>73</v>
       </c>
@@ -3341,34 +3503,590 @@
       <c r="C1" t="s">
         <v>74</v>
       </c>
+      <c r="D1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" t="s">
+        <v>54</v>
+      </c>
       <c r="G1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" t="s">
         <v>71</v>
       </c>
       <c r="I1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="K1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L1" t="s">
+        <v>114</v>
+      </c>
+      <c r="N1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
         <v>75</v>
       </c>
       <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J2">
+        <f>COUNTA(A2:A22) + 0.5 * COUNTA(H2:H22) + 0.4 * COUNTA(G2:G22) + 0.25 * COUNTA(F2:F22)</f>
+        <v>13</v>
+      </c>
+      <c r="K2">
+        <f>COUNTA(A2:A22) + 0.5 * COUNTA(H2:H22) + 0.5 * COUNTA(G2:G22) + 0.5 * COUNTA(F2:F22)</f>
+        <v>13</v>
+      </c>
+      <c r="L2">
+        <f>COUNTA(A2:A22) + 0.5 * COUNTA(H2:H22)</f>
+        <v>13</v>
+      </c>
+      <c r="O2">
         <v>8</v>
       </c>
-      <c r="G2" t="s">
+      <c r="P2">
+        <v>9</v>
+      </c>
+      <c r="Q2">
+        <v>10</v>
+      </c>
+      <c r="R2">
+        <v>11</v>
+      </c>
+      <c r="S2">
+        <v>12</v>
+      </c>
+      <c r="T2">
+        <v>13</v>
+      </c>
+      <c r="U2">
+        <v>14</v>
+      </c>
+      <c r="V2">
+        <v>15</v>
+      </c>
+      <c r="W2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>112</v>
+      </c>
+      <c r="I3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N3" t="s">
+        <v>92</v>
+      </c>
+      <c r="O3">
+        <v>4</v>
+      </c>
+      <c r="P3">
+        <v>3</v>
+      </c>
+      <c r="S3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="16">
+        <v>0.3125</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q4">
+        <v>3</v>
+      </c>
+      <c r="R4">
+        <v>3</v>
+      </c>
+      <c r="T4">
+        <v>2</v>
+      </c>
+      <c r="U4">
+        <v>2</v>
+      </c>
+      <c r="V4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="16">
+        <v>0.32291666666666669</v>
+      </c>
+      <c r="I5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I6" t="s">
+        <v>100</v>
+      </c>
+      <c r="N6" t="s">
+        <v>94</v>
+      </c>
+      <c r="O6">
+        <f>IF(O3 &gt; 0, (O3)*(O3-1)/2 * (O2/O3), 0)</f>
+        <v>12</v>
+      </c>
+      <c r="P6">
+        <f t="shared" ref="P6:T6" si="0">IF(P3 &gt; 0, (P3)*(P3-1)/2 * (P2/P3), 0)</f>
+        <v>9</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <f t="shared" ref="U6:V6" si="1">IF(U3 &gt; 0, (U3)*(U3-1)/2 * (U2/U3), 0)</f>
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="I7" t="s">
+        <v>109</v>
+      </c>
+      <c r="N7" t="s">
+        <v>95</v>
+      </c>
+      <c r="O7">
+        <f t="shared" ref="O7:P7" si="2">IF(O4&gt;0,O4 * O2 / 2, 0)</f>
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <f>IF(Q4&gt;0,Q4 * Q2 / 2, 0)</f>
+        <v>15</v>
+      </c>
+      <c r="R7">
+        <f t="shared" ref="R7:V7" si="3">IF(R4&gt;0,R4 * R2 / 2, 0)</f>
+        <v>16.5</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="16">
+        <v>0.32291666666666669</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" t="s">
+        <v>112</v>
+      </c>
+      <c r="N9" t="s">
+        <v>96</v>
+      </c>
+      <c r="O9">
+        <v>5</v>
+      </c>
+      <c r="P9">
+        <v>6</v>
+      </c>
+      <c r="Q9">
+        <v>6</v>
+      </c>
+      <c r="R9">
+        <v>6</v>
+      </c>
+      <c r="S9">
+        <v>8</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="N10" t="s">
+        <v>102</v>
+      </c>
+      <c r="T10">
+        <v>10</v>
+      </c>
+      <c r="U10">
+        <v>10</v>
+      </c>
+      <c r="V10">
+        <v>10</v>
+      </c>
+      <c r="W10">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="N11" t="s">
+        <v>115</v>
+      </c>
+      <c r="T11">
+        <v>13</v>
+      </c>
+      <c r="U11">
+        <v>13</v>
+      </c>
+      <c r="V11">
+        <v>13</v>
+      </c>
+      <c r="W11">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="I2">
-        <f>COUNTA(A2:A22) + 0.5 * COUNTA(G2:G22)</f>
+      <c r="D13" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="N13" t="s">
+        <v>97</v>
+      </c>
+      <c r="O13">
+        <f>O6 + O7 + O9</f>
+        <v>17</v>
+      </c>
+      <c r="P13">
+        <f>P6 + P7 + P9</f>
+        <v>15</v>
+      </c>
+      <c r="Q13">
+        <f>Q6 + Q7 + Q9</f>
+        <v>21</v>
+      </c>
+      <c r="R13">
+        <f>R6 + R7 + R9</f>
+        <v>22.5</v>
+      </c>
+      <c r="S13">
+        <f>S6 + S7 + S9</f>
+        <v>20</v>
+      </c>
+      <c r="T13">
+        <f>T6 + T7 + T9 + T11</f>
+        <v>26</v>
+      </c>
+      <c r="U13">
+        <f t="shared" ref="U13:W13" si="4">U6 + U7 + U9 + U11</f>
+        <v>27</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="4"/>
+        <v>28</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="4"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="K14" t="s">
+        <v>37</v>
+      </c>
+      <c r="L14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="K15">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="G3" t="s">
+      <c r="L15">
         <v>20</v>
+      </c>
+      <c r="N15" t="s">
+        <v>99</v>
+      </c>
+      <c r="O15">
+        <f>O13 * ($L$15 / 60) / $K$15</f>
+        <v>2.833333333333333</v>
+      </c>
+      <c r="P15">
+        <f t="shared" ref="P15:V15" si="5">P13 * ($L$15 / 60) / $K$15</f>
+        <v>2.5</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="5"/>
+        <v>3.5</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="5"/>
+        <v>3.75</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="5"/>
+        <v>3.333333333333333</v>
+      </c>
+      <c r="T15">
+        <f>T13 * ($L$15 / 60) / $K$15</f>
+        <v>4.333333333333333</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="5"/>
+        <v>4.5</v>
+      </c>
+      <c r="V15">
+        <f t="shared" si="5"/>
+        <v>4.6666666666666661</v>
+      </c>
+      <c r="W15">
+        <f t="shared" ref="W15" si="6">W13 * ($L$15 / 60) / $K$15</f>
+        <v>5.1666666666666661</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="K16" t="s">
+        <v>106</v>
+      </c>
+      <c r="L16" s="15">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="17" spans="10:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="J17" t="s">
+        <v>107</v>
+      </c>
+      <c r="N17" t="s">
+        <v>110</v>
+      </c>
+      <c r="O17">
+        <f t="shared" ref="O17:S17" si="7">($L$18 * (O6 + O7) + (O9 + O11) * $L$15) / ($K$15 * 60)</f>
+        <v>2.2333333333333334</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="7"/>
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="7"/>
+        <v>2.75</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="7"/>
+        <v>2.9249999999999998</v>
+      </c>
+      <c r="S17">
+        <f t="shared" si="7"/>
+        <v>2.7333333333333334</v>
+      </c>
+      <c r="T17">
+        <f>($L$18 * (T6 + T7) + (T9 + T11) * $L$15) / ($K$15 * 60)</f>
+        <v>3.6833333333333331</v>
+      </c>
+      <c r="U17">
+        <f t="shared" ref="U17:W17" si="8">($L$18 * (U6 + U7) + (U9 + U11) * $L$15) / ($K$15 * 60)</f>
+        <v>3.8</v>
+      </c>
+      <c r="V17">
+        <f t="shared" si="8"/>
+        <v>3.9166666666666665</v>
+      </c>
+      <c r="W17">
+        <f t="shared" si="8"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="18" spans="10:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="L18">
+        <f>L15 * (L16 * J18/6 + (1-L16))</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="10:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="N20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="10:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="N21" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="10:23" x14ac:dyDescent="0.55000000000000004">
+      <c r="N22" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated for the final crokinole
</commit_message>
<xml_diff>
--- a/static/jpFlicksSeason2.xlsx
+++ b/static/jpFlicksSeason2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1075" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EE9663C-5C1F-485F-A47E-524B0EA66088}"/>
+  <xr:revisionPtr revIDLastSave="1082" documentId="8_{867DBCD6-7AF9-4EBF-899F-19C6CCA2DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92C4A622-BF39-434B-9684-DADBC5BCB317}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="6" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{F2CC4DDF-27B6-4D19-B743-3CECDC910C25}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeGames" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="GameCalculator" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1265,10 +1266,10 @@
       </c>
       <c r="K2" s="4" t="str">
         <f>IF(OR(B11 = "UNPLAYED", B11 = "XXX"), B11, IF(B11 = "F", "-F", IF(B11 = "-F", "F", -1*B11)))</f>
-        <v>UNPLAYED</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+        <v>F</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -1347,7 +1348,7 @@
       </c>
       <c r="J4" s="4" t="str">
         <f>IF(OR(D10 = "UNPLAYED", D10 = "XXX"), D10, IF(D10 = "F", "-F", IF(D10 = "-F", "F", -1*D10)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="K4" s="4" t="str">
         <f>IF(OR(D11 = "UNPLAYED", D11 = "XXX"), D11, IF(D11 = "F", "-F", IF(D11 = "-F", "F", -1*D11)))</f>
@@ -1355,7 +1356,7 @@
       </c>
       <c r="O4" s="4"/>
     </row>
-    <row r="5" spans="1:17" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:17" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A5" s="9" t="s">
         <v>48</v>
       </c>
@@ -1397,7 +1398,7 @@
       </c>
       <c r="O5" s="4"/>
     </row>
-    <row r="6" spans="1:17" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:17" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A6" s="9" t="s">
         <v>47</v>
       </c>
@@ -1566,7 +1567,7 @@
         <v>75</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>3</v>
@@ -1598,8 +1599,8 @@
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>4</v>
+      <c r="B11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>70</v>
@@ -1739,7 +1740,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:12" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A2" s="9" t="s">
         <v>24</v>
       </c>
@@ -1783,7 +1784,7 @@
         <v>F</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:12" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -1868,7 +1869,7 @@
         <v>XXX</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:12" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A5" s="9" t="s">
         <v>48</v>
       </c>
@@ -1909,7 +1910,7 @@
         <v>F</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="25.8" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:12" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A6" s="9" t="s">
         <v>47</v>
       </c>
@@ -1973,7 +1974,7 @@
       </c>
       <c r="H7" s="4" t="str">
         <f>IF(OR(G8 = "UNPLAYED", G8 = "XXX"), G8, IF(G8 = "F", "-F", IF(G8 = "-F", "F", -1*G8)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="I7" s="4" t="str">
         <f>IF(OR(G9 = "UNPLAYED", G9 = "XXX"), G9, IF(G9 = "F", "-F", IF(G9 = "-F", "F", -1*G9)))</f>
@@ -1981,7 +1982,7 @@
       </c>
       <c r="J7" s="4" t="str">
         <f>IF(OR(G10 = "UNPLAYED", G10 = "XXX"), G10, IF(G10 = "F", "-F", IF(G10 = "-F", "F", -1*G10)))</f>
-        <v>UNPLAYED</v>
+        <v>-F</v>
       </c>
       <c r="K7" s="4" t="str">
         <f>IF(OR(G11 = "UNPLAYED", G11 = "XXX"), G11, IF(G11 = "F", "-F", IF(G11 = "-F", "F", -1*G11)))</f>
@@ -2008,14 +2009,14 @@
         <v>70</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>3</v>
       </c>
       <c r="I8" s="4" t="str">
         <f>IF(OR(H9 = "UNPLAYED", H9 = "XXX"), H9, IF(H9 = "F", "-F", IF(H9 = "-F", "F", -1*H9)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="J8" s="4" t="str">
         <f>IF(OR(H10 = "UNPLAYED", H10 = "XXX"), H10, IF(H10 = "F", "-F", IF(H10 = "-F", "F", -1*H10)))</f>
@@ -2023,7 +2024,7 @@
       </c>
       <c r="K8" s="4" t="str">
         <f>IF(OR(H11 = "UNPLAYED", H11 = "XXX"), H11, IF(H11 = "F", "-F", IF(H11 = "-F", "F", -1*H11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="25.5" x14ac:dyDescent="0.55000000000000004">
@@ -2048,8 +2049,8 @@
       <c r="G9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>4</v>
+      <c r="H9" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>3</v>
@@ -2084,7 +2085,7 @@
         <v>100</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>69</v>
@@ -2097,11 +2098,11 @@
       </c>
       <c r="K10" s="4" t="str">
         <f>IF(OR(J11 = "UNPLAYED", J11 = "XXX"), J11, IF(J11 = "F", "-F", IF(J11 = "-F", "F", -1*J11)))</f>
-        <v>UNPLAYED</v>
+        <v>F</v>
       </c>
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:12" ht="25.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>56</v>
       </c>
@@ -2123,14 +2124,14 @@
       <c r="G11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>4</v>
+      <c r="H11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="I11" s="3">
         <v>0</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>4</v>
+      <c r="J11" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>3</v>

</xml_diff>